<commit_message>
Fix: admin badge color matches academy, archived video preview, updated XLSX template
</commit_message>
<xml_diff>
--- a/public/templates/Users_example.xlsx
+++ b/public/templates/Users_example.xlsx
@@ -4,6 +4,7 @@
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
     <sheet name="Usuarios" sheetId="1" r:id="rId1"/>
+    <sheet name="Clases" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
 </file>
@@ -564,4 +565,64 @@
     <ignoredError numberStoredAsText="1" sqref="A1:E9"/>
   </ignoredErrors>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:C4"/>
+  <cols>
+    <col min="1" max="1" width="24.83203125" customWidth="1"/>
+    <col min="2" max="2" width="16.83203125" customWidth="1"/>
+    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="str">
+        <v>nombre</v>
+      </c>
+      <c r="B1" t="str">
+        <v>precioMensual</v>
+      </c>
+      <c r="C1" t="str">
+        <v>pagoUnico</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="str">
+        <v>Matemáticas 1</v>
+      </c>
+      <c r="B2" t="str">
+        <v>50</v>
+      </c>
+      <c r="C2" t="str">
+        <v/>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="str">
+        <v>Inglés B2</v>
+      </c>
+      <c r="B3" t="str">
+        <v/>
+      </c>
+      <c r="C3" t="str">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="str">
+        <v>Ciencias</v>
+      </c>
+      <c r="B4" t="str">
+        <v>40</v>
+      </c>
+      <c r="C4" t="str">
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <ignoredErrors>
+    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fix: admin Pagos badge green, class sheet redesign (startDate+price+teacher), VideoCard inline player
</commit_message>
<xml_diff>
--- a/public/templates/Users_example.xlsx
+++ b/public/templates/Users_example.xlsx
@@ -569,11 +569,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C4"/>
+  <dimension ref="A1:E4"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
-    <col min="2" max="2" width="16.83203125" customWidth="1"/>
-    <col min="3" max="3" width="12.83203125" customWidth="1"/>
+    <col min="2" max="2" width="14.83203125" customWidth="1"/>
+    <col min="3" max="3" width="10.83203125" customWidth="1"/>
+    <col min="4" max="4" width="12.83203125" customWidth="1"/>
+    <col min="5" max="5" width="30.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -581,10 +583,16 @@
         <v>nombre</v>
       </c>
       <c r="B1" t="str">
-        <v>precioMensual</v>
+        <v>fechaInicio</v>
       </c>
       <c r="C1" t="str">
-        <v>pagoUnico</v>
+        <v>precio</v>
+      </c>
+      <c r="D1" t="str">
+        <v>tipoPrecio</v>
+      </c>
+      <c r="E1" t="str">
+        <v>profesorEmail</v>
       </c>
     </row>
     <row r="2">
@@ -592,10 +600,16 @@
         <v>Matemáticas 1</v>
       </c>
       <c r="B2" t="str">
+        <v>01/09/2026</v>
+      </c>
+      <c r="C2" t="str">
         <v>50</v>
       </c>
-      <c r="C2" t="str">
-        <v/>
+      <c r="D2" t="str">
+        <v>MENSUAL</v>
+      </c>
+      <c r="E2" t="str">
+        <v>miguel.ruiz@ejemplo.com</v>
       </c>
     </row>
     <row r="3">
@@ -603,10 +617,16 @@
         <v>Inglés B2</v>
       </c>
       <c r="B3" t="str">
-        <v/>
+        <v>15/09/2026</v>
       </c>
       <c r="C3" t="str">
         <v>200</v>
+      </c>
+      <c r="D3" t="str">
+        <v>UNICO</v>
+      </c>
+      <c r="E3" t="str">
+        <v>sofia.moreno@ejemplo.com</v>
       </c>
     </row>
     <row r="4">
@@ -614,15 +634,21 @@
         <v>Ciencias</v>
       </c>
       <c r="B4" t="str">
+        <v>01/09/2026</v>
+      </c>
+      <c r="C4" t="str">
         <v>40</v>
       </c>
-      <c r="C4" t="str">
-        <v/>
+      <c r="D4" t="str">
+        <v>MENSUAL</v>
+      </c>
+      <c r="E4" t="str">
+        <v>sofia.moreno@ejemplo.com</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add universidad, carrera, maxStudents, descripcion, whatsapp to class migration sheet
</commit_message>
<xml_diff>
--- a/public/templates/Users_example.xlsx
+++ b/public/templates/Users_example.xlsx
@@ -569,13 +569,18 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:J4"/>
   <cols>
     <col min="1" max="1" width="24.83203125" customWidth="1"/>
     <col min="2" max="2" width="14.83203125" customWidth="1"/>
     <col min="3" max="3" width="10.83203125" customWidth="1"/>
     <col min="4" max="4" width="12.83203125" customWidth="1"/>
     <col min="5" max="5" width="30.83203125" customWidth="1"/>
+    <col min="6" max="6" width="36.83203125" customWidth="1"/>
+    <col min="7" max="7" width="16.83203125" customWidth="1"/>
+    <col min="8" max="8" width="16.83203125" customWidth="1"/>
+    <col min="9" max="9" width="14.83203125" customWidth="1"/>
+    <col min="10" max="10" width="40.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -594,6 +599,21 @@
       <c r="E1" t="str">
         <v>profesorEmail</v>
       </c>
+      <c r="F1" t="str">
+        <v>descripcion</v>
+      </c>
+      <c r="G1" t="str">
+        <v>universidad</v>
+      </c>
+      <c r="H1" t="str">
+        <v>carrera</v>
+      </c>
+      <c r="I1" t="str">
+        <v>maxEstudiantes</v>
+      </c>
+      <c r="J1" t="str">
+        <v>whatsapp</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -611,6 +631,21 @@
       <c r="E2" t="str">
         <v>miguel.ruiz@ejemplo.com</v>
       </c>
+      <c r="F2" t="str">
+        <v>Álgebra y cálculo básico</v>
+      </c>
+      <c r="G2" t="str">
+        <v>UCM</v>
+      </c>
+      <c r="H2" t="str">
+        <v>Ingeniería</v>
+      </c>
+      <c r="I2" t="str">
+        <v>30</v>
+      </c>
+      <c r="J2" t="str">
+        <v/>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -628,6 +663,21 @@
       <c r="E3" t="str">
         <v>sofia.moreno@ejemplo.com</v>
       </c>
+      <c r="F3" t="str">
+        <v>Inglés nivel B2</v>
+      </c>
+      <c r="G3" t="str">
+        <v/>
+      </c>
+      <c r="H3" t="str">
+        <v/>
+      </c>
+      <c r="I3" t="str">
+        <v>20</v>
+      </c>
+      <c r="J3" t="str">
+        <v>https://chat.whatsapp.com/ejemplo</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -645,10 +695,25 @@
       <c r="E4" t="str">
         <v>sofia.moreno@ejemplo.com</v>
       </c>
+      <c r="F4" t="str">
+        <v/>
+      </c>
+      <c r="G4" t="str">
+        <v>UAM</v>
+      </c>
+      <c r="H4" t="str">
+        <v>Biología</v>
+      </c>
+      <c r="I4" t="str">
+        <v/>
+      </c>
+      <c r="J4" t="str">
+        <v/>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E4"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:J4"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>